<commit_message>
feat: rebalance survival economy and add scavenger crates
</commit_message>
<xml_diff>
--- a/docs/balance/LOTM_MC_Addon_数值平衡总表.xlsx
+++ b/docs/balance/LOTM_MC_Addon_数值平衡总表.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览与口径" sheetId="1" r:id="R3043cdef1e5a464b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枪械武器" sheetId="2" r:id="Rd57f47cf2bba47a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="护甲与装备" sheetId="3" r:id="Rdc5bbf56d2c6444d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蓝图" sheetId="4" r:id="R00a95b81925a4cc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="半成品与材料" sheetId="5" r:id="R16ca79b3a1a54c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配方明细" sheetId="6" r:id="Rf969628c606446e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原版材料折算" sheetId="7" r:id="R0bf12ab23c4847d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="载具属性" sheetId="8" r:id="R2a1a870b16ca4197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="载具配方" sheetId="9" r:id="Rea26bdbe1d4b4fbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物与Boss" sheetId="10" r:id="R1f11fd6945794ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落明细" sheetId="11" r:id="R5d3bfa3912494480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="副本与奖池" sheetId="12" r:id="Ra67c72c4dcc14dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平衡仪表盘" sheetId="13" r:id="Rf93a8707f9794c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览与口径" sheetId="1" r:id="R26948e0d874d4f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枪械武器" sheetId="2" r:id="Rfb4b055cc38c4ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="护甲与装备" sheetId="3" r:id="Rd4f015da7c2749bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="蓝图" sheetId="4" r:id="Re0f97d36b7324963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="半成品与材料" sheetId="5" r:id="Ra7fc394e845d4f5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配方明细" sheetId="6" r:id="R493790c05b1c4722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原版材料折算" sheetId="7" r:id="R3bfed3a274d8416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="载具属性" sheetId="8" r:id="R4d825341b1f44f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="载具配方" sheetId="9" r:id="R38a7867c0e774b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物与Boss" sheetId="10" r:id="R3422f047c547473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掉落明细" sheetId="11" r:id="R9f57615fbe74410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="副本与奖池" sheetId="12" r:id="Ra590c852887146ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="平衡仪表盘" sheetId="13" r:id="R3d142b319b444b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MVP经济配置" sheetId="14" r:id="R61ee67f79db54026"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,13 +26,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0%"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="0.00%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -98,8 +101,32 @@
       <x:color rgb="FF172B4D"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF44546A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -141,8 +168,33 @@
         <x:fgColor rgb="FFD45D5D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF14233B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2B6CB0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2A9D8F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="6">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -162,11 +214,39 @@
         <x:color rgb="FFE6ECF2"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE6D18A"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE6D18A"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE6D18A"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE6D18A"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="96">
+  <x:cellXfs count="131">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -411,6 +491,81 @@
     <x:xf numFmtId="201" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -578,7 +733,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R67b6234021494d63"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb424c364266a4cb6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1140,7 +1295,7 @@
         <x:v>数据快照</x:v>
       </x:c>
       <x:c r="B5" s="48" t="str">
-        <x:v>Git commit f383d05769b1a71b5bb939f506c57b7c6821261d</x:v>
+        <x:v>工作树版本：MVP 单金币经济改版（尚未上传 GitHub）</x:v>
       </x:c>
       <x:c r="C5" s="48"/>
       <x:c r="D5" s="48" t="str">
@@ -1359,17 +1514,17 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="48" t="str">
-        <x:v>奖池概率</x:v>
+        <x:v>本次更新</x:v>
       </x:c>
       <x:c r="B17" s="48" t="str">
-        <x:v>权重÷权重合计；工作表中用公式计算，便于修改权重试算</x:v>
-      </x:c>
-      <x:c r="C17" s="48" t="str"/>
-      <x:c r="D17" s="48" t="str"/>
-      <x:c r="E17" s="48" t="str"/>
-      <x:c r="F17" s="48" t="str"/>
-      <x:c r="G17" s="48" t="str"/>
-      <x:c r="H17" s="48" t="str"/>
+        <x:v>双奖池 20/30 抽保底、神话密钥、日常/副本金币、分层掉落、载具与限定蓝图来源；详见“MVP经济配置”</x:v>
+      </x:c>
+      <x:c r="C17" s="48"/>
+      <x:c r="D17" s="48"/>
+      <x:c r="E17" s="48"/>
+      <x:c r="F17" s="48"/>
+      <x:c r="G17" s="48"/>
+      <x:c r="H17" s="48"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2369,7 +2524,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78fa9706b77847b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02d2ba166fad4091"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6234,7 +6389,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ee9f2c14e3145de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14d4ff3419294593"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7189,7 +7344,1623 @@
     <x:mergeCell ref="A2:N2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4481337dfe8a4a31"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a1a383add134215"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="130" t="str">
+        <x:v>LOTM-MC · MVP 单金币经济配置</x:v>
+      </x:c>
+      <x:c r="B1" s="130"/>
+      <x:c r="C1" s="130"/>
+      <x:c r="D1" s="130"/>
+      <x:c r="E1" s="130"/>
+      <x:c r="F1" s="130"/>
+      <x:c r="G1" s="130"/>
+      <x:c r="H1" s="130"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="101" t="str">
+        <x:v>唯一货币金币；研究券/声望/维修币/阵营条件均不引入。黄色数值为可调参数，概率与保底总价使用公式。</x:v>
+      </x:c>
+      <x:c r="B2" s="101"/>
+      <x:c r="C2" s="101"/>
+      <x:c r="D2" s="101"/>
+      <x:c r="E2" s="101"/>
+      <x:c r="F2" s="101"/>
+      <x:c r="G2" s="101"/>
+      <x:c r="H2" s="101"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="106" t="str">
+        <x:v>关键目标</x:v>
+      </x:c>
+      <x:c r="B4" s="106" t="str">
+        <x:v>数值</x:v>
+      </x:c>
+      <x:c r="C4" s="106" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+      <x:c r="D4" s="106" t="str"/>
+      <x:c r="E4" s="106" t="str"/>
+      <x:c r="F4" s="106" t="str"/>
+      <x:c r="G4" s="106" t="str"/>
+      <x:c r="H4" s="106" t="str"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="125" t="str">
+        <x:v>正常活跃日收入</x:v>
+      </x:c>
+      <x:c r="B5" s="126" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="C5" s="125" t="str">
+        <x:v>60–120 分钟基准</x:v>
+      </x:c>
+      <x:c r="D5" s="125" t="str"/>
+      <x:c r="E5" s="125" t="str"/>
+      <x:c r="F5" s="125" t="str"/>
+      <x:c r="G5" s="125" t="str"/>
+      <x:c r="H5" s="125" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="125" t="str">
+        <x:v>Epic 最坏保底总价</x:v>
+      </x:c>
+      <x:c r="B6" s="126" t="n">
+        <x:f>D11</x:f>
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="C6" s="125" t="str">
+        <x:v>20 抽</x:v>
+      </x:c>
+      <x:c r="D6" s="125" t="str"/>
+      <x:c r="E6" s="125" t="str"/>
+      <x:c r="F6" s="125" t="str"/>
+      <x:c r="G6" s="125" t="str"/>
+      <x:c r="H6" s="125" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="125" t="str">
+        <x:v>Legendary 最坏保底总价</x:v>
+      </x:c>
+      <x:c r="B7" s="126" t="n">
+        <x:f>D12</x:f>
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="C7" s="125" t="str">
+        <x:v>30 抽</x:v>
+      </x:c>
+      <x:c r="D7" s="125" t="str"/>
+      <x:c r="E7" s="125" t="str"/>
+      <x:c r="F7" s="125" t="str"/>
+      <x:c r="G7" s="125" t="str"/>
+      <x:c r="H7" s="125" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="125" t="str">
+        <x:v>Legendary 第一期</x:v>
+      </x:c>
+      <x:c r="B8" s="126" t="str">
+        <x:v>HK MP7 暴走狂潮</x:v>
+      </x:c>
+      <x:c r="C8" s="125" t="str">
+        <x:v>管理员可在 SAPI 后台切换</x:v>
+      </x:c>
+      <x:c r="D8" s="125" t="str"/>
+      <x:c r="E8" s="125" t="str"/>
+      <x:c r="F8" s="125" t="str"/>
+      <x:c r="G8" s="125" t="str"/>
+      <x:c r="H8" s="125" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="125" t="str"/>
+      <x:c r="B9" s="125" t="str"/>
+      <x:c r="C9" s="125" t="str"/>
+      <x:c r="D9" s="125" t="str"/>
+      <x:c r="E9" s="125" t="str"/>
+      <x:c r="F9" s="125" t="str"/>
+      <x:c r="G9" s="125" t="str"/>
+      <x:c r="H9" s="125" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="111" t="str">
+        <x:v>金币抽奖池</x:v>
+      </x:c>
+      <x:c r="B10" s="111" t="str">
+        <x:v>单抽</x:v>
+      </x:c>
+      <x:c r="C10" s="111" t="str">
+        <x:v>硬保底次数</x:v>
+      </x:c>
+      <x:c r="D10" s="111" t="str">
+        <x:v>最坏保底总价</x:v>
+      </x:c>
+      <x:c r="E10" s="111" t="str">
+        <x:v>完整目标基础概率</x:v>
+      </x:c>
+      <x:c r="F10" s="111" t="str">
+        <x:v>保底内容</x:v>
+      </x:c>
+      <x:c r="G10" s="111" t="str">
+        <x:v>十连价</x:v>
+      </x:c>
+      <x:c r="H10" s="111" t="str">
+        <x:v>演出</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="125" t="str">
+        <x:v>Epic 高级军备箱</x:v>
+      </x:c>
+      <x:c r="B11" s="126" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="C11" s="126" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D11" s="126" t="n">
+        <x:f>B11*C11</x:f>
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="E11" s="127" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="F11" s="125" t="str">
+        <x:v>随机限定 Epic 蓝图</x:v>
+      </x:c>
+      <x:c r="G11" s="125" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="H11" s="125" t="str">
+        <x:v>聊天+粒子+分阶段音效</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="125" t="str">
+        <x:v>Legendary 限定军备箱</x:v>
+      </x:c>
+      <x:c r="B12" s="126" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="C12" s="126" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D12" s="126" t="n">
+        <x:f>B12*C12</x:f>
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="E12" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F12" s="125" t="str">
+        <x:v>当期唯一 UP 蓝图</x:v>
+      </x:c>
+      <x:c r="G12" s="125" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="H12" s="125" t="str">
+        <x:v>稀有度差异音效；不占 Action Bar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="125" t="str"/>
+      <x:c r="B13" s="125" t="str"/>
+      <x:c r="C13" s="125" t="str"/>
+      <x:c r="D13" s="125" t="str"/>
+      <x:c r="E13" s="125" t="str"/>
+      <x:c r="F13" s="125" t="str"/>
+      <x:c r="G13" s="125" t="str"/>
+      <x:c r="H13" s="125" t="str"/>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="111" t="str">
+        <x:v>Epic 限定蓝图</x:v>
+      </x:c>
+      <x:c r="B14" s="111" t="str">
+        <x:v>名称</x:v>
+      </x:c>
+      <x:c r="C14" s="111" t="str">
+        <x:v>池内权重</x:v>
+      </x:c>
+      <x:c r="D14" s="111" t="str">
+        <x:v>实际概率</x:v>
+      </x:c>
+      <x:c r="E14" s="111" t="str">
+        <x:v>保底候选</x:v>
+      </x:c>
+      <x:c r="F14" s="111" t="str">
+        <x:v>玩家合成</x:v>
+      </x:c>
+      <x:c r="G14" s="111" t="str">
+        <x:v>NPC 指定价</x:v>
+      </x:c>
+      <x:c r="H14" s="111" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="125" t="str">
+        <x:v>test_gun:blueprint_pkm</x:v>
+      </x:c>
+      <x:c r="B15" s="125" t="str">
+        <x:v>PKM 烈焰重机枪</x:v>
+      </x:c>
+      <x:c r="C15" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="127" t="n">
+        <x:f>C15/SUM($C$15:$C$19)*5%</x:f>
+        <x:v>0.010000000000000002</x:v>
+      </x:c>
+      <x:c r="E15" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F15" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="G15" s="126" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="H15" s="125" t="str">
+        <x:v>Epic 池/高级军备商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="125" t="str">
+        <x:v>test_gun:blueprint_usas12</x:v>
+      </x:c>
+      <x:c r="B16" s="125" t="str">
+        <x:v>USAS-12 嗜血狂潮</x:v>
+      </x:c>
+      <x:c r="C16" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="127" t="n">
+        <x:f>C16/SUM($C$15:$C$19)*5%</x:f>
+        <x:v>0.010000000000000002</x:v>
+      </x:c>
+      <x:c r="E16" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F16" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="G16" s="126" t="n">
+        <x:v>32000</x:v>
+      </x:c>
+      <x:c r="H16" s="125" t="str">
+        <x:v>Epic 池/高级军备商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="125" t="str">
+        <x:v>test_gun:blueprint_m1014_ward</x:v>
+      </x:c>
+      <x:c r="B17" s="125" t="str">
+        <x:v>M1014 泰坦壁垒</x:v>
+      </x:c>
+      <x:c r="C17" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="127" t="n">
+        <x:f>C17/SUM($C$15:$C$19)*5%</x:f>
+        <x:v>0.010000000000000002</x:v>
+      </x:c>
+      <x:c r="E17" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F17" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="G17" s="126" t="n">
+        <x:v>28000</x:v>
+      </x:c>
+      <x:c r="H17" s="125" t="str">
+        <x:v>Epic 池/高级军备商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="125" t="str">
+        <x:v>test_gun:blueprint_flash_shield</x:v>
+      </x:c>
+      <x:c r="B18" s="125" t="str">
+        <x:v>G52 战术闪光盾</x:v>
+      </x:c>
+      <x:c r="C18" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="127" t="n">
+        <x:f>C18/SUM($C$15:$C$19)*5%</x:f>
+        <x:v>0.010000000000000002</x:v>
+      </x:c>
+      <x:c r="E18" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F18" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="G18" s="126" t="n">
+        <x:v>26000</x:v>
+      </x:c>
+      <x:c r="H18" s="125" t="str">
+        <x:v>Epic 池/高级军备商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="125" t="str">
+        <x:v>test_gun:blueprint_titan_chest</x:v>
+      </x:c>
+      <x:c r="B19" s="125" t="str">
+        <x:v>泰坦动力外骨骼</x:v>
+      </x:c>
+      <x:c r="C19" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="127" t="n">
+        <x:f>C19/SUM($C$15:$C$19)*5%</x:f>
+        <x:v>0.010000000000000002</x:v>
+      </x:c>
+      <x:c r="E19" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="F19" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="G19" s="126" t="n">
+        <x:v>36000</x:v>
+      </x:c>
+      <x:c r="H19" s="125" t="str">
+        <x:v>Epic 池/高级军备商</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="125" t="str"/>
+      <x:c r="B20" s="125" t="str"/>
+      <x:c r="C20" s="125" t="str"/>
+      <x:c r="D20" s="125" t="str"/>
+      <x:c r="E20" s="125" t="str"/>
+      <x:c r="F20" s="125" t="str"/>
+      <x:c r="G20" s="125" t="str"/>
+      <x:c r="H20" s="125" t="str"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="111" t="str">
+        <x:v>Legendary 候选</x:v>
+      </x:c>
+      <x:c r="B21" s="111" t="str">
+        <x:v>名称</x:v>
+      </x:c>
+      <x:c r="C21" s="111" t="str">
+        <x:v>第一期</x:v>
+      </x:c>
+      <x:c r="D21" s="111" t="str">
+        <x:v>当期入池</x:v>
+      </x:c>
+      <x:c r="E21" s="111" t="str">
+        <x:v>基础概率</x:v>
+      </x:c>
+      <x:c r="F21" s="111" t="str">
+        <x:v>30 抽保底</x:v>
+      </x:c>
+      <x:c r="G21" s="111" t="str">
+        <x:v>玩家合成</x:v>
+      </x:c>
+      <x:c r="H21" s="111" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="125" t="str">
+        <x:v>test_gun:blueprint_mp7</x:v>
+      </x:c>
+      <x:c r="B22" s="125" t="str">
+        <x:v>HK MP7 暴走狂潮</x:v>
+      </x:c>
+      <x:c r="C22" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="D22" s="125" t="str">
+        <x:v>是（默认）</x:v>
+      </x:c>
+      <x:c r="E22" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F22" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G22" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H22" s="125" t="str">
+        <x:v>Legendary 当期限定池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="125" t="str">
+        <x:v>test_gun:blueprint_mgl</x:v>
+      </x:c>
+      <x:c r="B23" s="125" t="str">
+        <x:v>MGL 自动榴弹炮</x:v>
+      </x:c>
+      <x:c r="C23" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D23" s="125" t="str">
+        <x:v>管理员切换后</x:v>
+      </x:c>
+      <x:c r="E23" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F23" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G23" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H23" s="125" t="str">
+        <x:v>Legendary 当期限定池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="125" t="str">
+        <x:v>test_gun:blueprint_arc</x:v>
+      </x:c>
+      <x:c r="B24" s="125" t="str">
+        <x:v>Tesla 高能电弧风暴</x:v>
+      </x:c>
+      <x:c r="C24" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D24" s="125" t="str">
+        <x:v>管理员切换后</x:v>
+      </x:c>
+      <x:c r="E24" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F24" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G24" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H24" s="125" t="str">
+        <x:v>Legendary 当期限定池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="125" t="str">
+        <x:v>test_gun:blueprint_jetpack</x:v>
+      </x:c>
+      <x:c r="B25" s="125" t="str">
+        <x:v>战术离子喷气背包</x:v>
+      </x:c>
+      <x:c r="C25" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D25" s="125" t="str">
+        <x:v>管理员切换后</x:v>
+      </x:c>
+      <x:c r="E25" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F25" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G25" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H25" s="125" t="str">
+        <x:v>Legendary 当期限定池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A26" s="125" t="str">
+        <x:v>test_gun:blueprint_ak47_commander</x:v>
+      </x:c>
+      <x:c r="B26" s="125" t="str">
+        <x:v>AK-47 战术指挥官</x:v>
+      </x:c>
+      <x:c r="C26" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D26" s="125" t="str">
+        <x:v>管理员切换后</x:v>
+      </x:c>
+      <x:c r="E26" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="F26" s="125" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="G26" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="H26" s="125" t="str">
+        <x:v>Legendary 当期限定池</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="125" t="str"/>
+      <x:c r="B27" s="125" t="str"/>
+      <x:c r="C27" s="125" t="str"/>
+      <x:c r="D27" s="125" t="str"/>
+      <x:c r="E27" s="125" t="str"/>
+      <x:c r="F27" s="125" t="str"/>
+      <x:c r="G27" s="125" t="str"/>
+      <x:c r="H27" s="125" t="str"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="111" t="str">
+        <x:v>神话补给密钥</x:v>
+      </x:c>
+      <x:c r="B28" s="111" t="str">
+        <x:v>用途</x:v>
+      </x:c>
+      <x:c r="C28" s="111" t="str">
+        <x:v>可合成</x:v>
+      </x:c>
+      <x:c r="D28" s="111" t="str">
+        <x:v>Epic 箱额外概率</x:v>
+      </x:c>
+      <x:c r="E28" s="111" t="str">
+        <x:v>Legendary 箱额外概率</x:v>
+      </x:c>
+      <x:c r="F28" s="111" t="str">
+        <x:v>Mythic 箱返还概率</x:v>
+      </x:c>
+      <x:c r="G28" s="111" t="str">
+        <x:v>金币奖池</x:v>
+      </x:c>
+      <x:c r="H28" s="111" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="125" t="str">
+        <x:v>daily:mythic_supply_key</x:v>
+      </x:c>
+      <x:c r="B29" s="125" t="str">
+        <x:v>开启神话物资箱并消耗 1 个</x:v>
+      </x:c>
+      <x:c r="C29" s="125" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="D29" s="127" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="E29" s="127" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="F29" s="127" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="G29" s="125" t="str">
+        <x:v>Epic/Legendary 均可出</x:v>
+      </x:c>
+      <x:c r="H29" s="125" t="str">
+        <x:v>旧版命名回响碎片兼容一次</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="125" t="str"/>
+      <x:c r="B30" s="125" t="str"/>
+      <x:c r="C30" s="125" t="str"/>
+      <x:c r="D30" s="125" t="str"/>
+      <x:c r="E30" s="125" t="str"/>
+      <x:c r="F30" s="125" t="str"/>
+      <x:c r="G30" s="125" t="str"/>
+      <x:c r="H30" s="125" t="str"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="111" t="str">
+        <x:v>每日委托</x:v>
+      </x:c>
+      <x:c r="B31" s="111" t="str">
+        <x:v>金币</x:v>
+      </x:c>
+      <x:c r="C31" s="111" t="str">
+        <x:v>每日数量</x:v>
+      </x:c>
+      <x:c r="D31" s="111" t="str">
+        <x:v>小计</x:v>
+      </x:c>
+      <x:c r="E31" s="111" t="str">
+        <x:v>统计规则</x:v>
+      </x:c>
+      <x:c r="F31" s="111" t="str"/>
+      <x:c r="G31" s="111" t="str"/>
+      <x:c r="H31" s="111" t="str"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="125" t="str">
+        <x:v>采集</x:v>
+      </x:c>
+      <x:c r="B32" s="126" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="C32" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D32" s="126" t="n">
+        <x:f>B32*C32</x:f>
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="E32" s="125" t="str">
+        <x:v>只计接取后背包正增量</x:v>
+      </x:c>
+      <x:c r="F32" s="125" t="str"/>
+      <x:c r="G32" s="125" t="str"/>
+      <x:c r="H32" s="125" t="str"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="125" t="str">
+        <x:v>击杀</x:v>
+      </x:c>
+      <x:c r="B33" s="126" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C33" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D33" s="126" t="n">
+        <x:f>B33*C33</x:f>
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="E33" s="125" t="str">
+        <x:v>按怪物层级/参与记录</x:v>
+      </x:c>
+      <x:c r="F33" s="125" t="str"/>
+      <x:c r="G33" s="125" t="str"/>
+      <x:c r="H33" s="125" t="str"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="125" t="str">
+        <x:v>动态事件</x:v>
+      </x:c>
+      <x:c r="B34" s="126" t="n">
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="C34" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D34" s="126" t="n">
+        <x:f>B34*C34</x:f>
+        <x:v>1100</x:v>
+      </x:c>
+      <x:c r="E34" s="125" t="str">
+        <x:v>完成任意动态事件</x:v>
+      </x:c>
+      <x:c r="F34" s="125" t="str"/>
+      <x:c r="G34" s="125" t="str"/>
+      <x:c r="H34" s="125" t="str"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="125" t="str">
+        <x:v>综合</x:v>
+      </x:c>
+      <x:c r="B35" s="126" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="C35" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D35" s="126" t="n">
+        <x:f>B35*C35</x:f>
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="E35" s="125" t="str">
+        <x:v>副本/制造/半成品/箱子/Boss</x:v>
+      </x:c>
+      <x:c r="F35" s="125" t="str"/>
+      <x:c r="G35" s="125" t="str"/>
+      <x:c r="H35" s="125" t="str"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="125" t="str">
+        <x:v>四项完成额外</x:v>
+      </x:c>
+      <x:c r="B36" s="126" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="C36" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D36" s="126" t="n">
+        <x:f>B36*C36</x:f>
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="E36" s="125" t="str">
+        <x:v>100 活跃领取</x:v>
+      </x:c>
+      <x:c r="F36" s="125" t="str"/>
+      <x:c r="G36" s="125" t="str"/>
+      <x:c r="H36" s="125" t="str"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="125" t="str">
+        <x:v>日常合计</x:v>
+      </x:c>
+      <x:c r="B37" s="126" t="str"/>
+      <x:c r="C37" s="126" t="str"/>
+      <x:c r="D37" s="126" t="n">
+        <x:f>SUM(D32:D36)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E37" s="125" t="str">
+        <x:v>目标 6000</x:v>
+      </x:c>
+      <x:c r="F37" s="125" t="str"/>
+      <x:c r="G37" s="125" t="str"/>
+      <x:c r="H37" s="125" t="str"/>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="125" t="str"/>
+      <x:c r="B38" s="125" t="str"/>
+      <x:c r="C38" s="125" t="str"/>
+      <x:c r="D38" s="125" t="str"/>
+      <x:c r="E38" s="125" t="str"/>
+      <x:c r="F38" s="125" t="str"/>
+      <x:c r="G38" s="125" t="str"/>
+      <x:c r="H38" s="125" t="str"/>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="111" t="str">
+        <x:v>副本难度</x:v>
+      </x:c>
+      <x:c r="B39" s="111" t="str">
+        <x:v>首次金币</x:v>
+      </x:c>
+      <x:c r="C39" s="111" t="str">
+        <x:v>重复金币</x:v>
+      </x:c>
+      <x:c r="D39" s="111" t="str">
+        <x:v>Epic 蓝图概率</x:v>
+      </x:c>
+      <x:c r="E39" s="111" t="str">
+        <x:v>第1–2次</x:v>
+      </x:c>
+      <x:c r="F39" s="111" t="str">
+        <x:v>第3–4次</x:v>
+      </x:c>
+      <x:c r="G39" s="111" t="str">
+        <x:v>第5次以后</x:v>
+      </x:c>
+      <x:c r="H39" s="111" t="str">
+        <x:v>蓝图范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="125" t="str">
+        <x:v>Normal</x:v>
+      </x:c>
+      <x:c r="B40" s="126" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="C40" s="126" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="D40" s="128" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="128" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F40" s="128" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G40" s="128" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H40" s="125" t="str">
+        <x:v>无</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="125" t="str">
+        <x:v>Hard</x:v>
+      </x:c>
+      <x:c r="B41" s="126" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="C41" s="126" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D41" s="128" t="n">
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="E41" s="128" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F41" s="128" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G41" s="128" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H41" s="125" t="str">
+        <x:v>可合成 Epic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="125" t="str">
+        <x:v>Nightmare</x:v>
+      </x:c>
+      <x:c r="B42" s="126" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C42" s="126" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="D42" s="128" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="E42" s="128" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F42" s="128" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G42" s="128" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H42" s="125" t="str">
+        <x:v>可合成 Epic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="125" t="str"/>
+      <x:c r="B43" s="125" t="str"/>
+      <x:c r="C43" s="125" t="str"/>
+      <x:c r="D43" s="125" t="str"/>
+      <x:c r="E43" s="125" t="str"/>
+      <x:c r="F43" s="125" t="str"/>
+      <x:c r="G43" s="125" t="str"/>
+      <x:c r="H43" s="125" t="str"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="111" t="str">
+        <x:v>怪物层级</x:v>
+      </x:c>
+      <x:c r="B44" s="111" t="str">
+        <x:v>主要原版掉落</x:v>
+      </x:c>
+      <x:c r="C44" s="111" t="str">
+        <x:v>半成品概率</x:v>
+      </x:c>
+      <x:c r="D44" s="111" t="str">
+        <x:v>完整 Epic 蓝图概率</x:v>
+      </x:c>
+      <x:c r="E44" s="111" t="str">
+        <x:v>Legendary</x:v>
+      </x:c>
+      <x:c r="F44" s="111" t="str">
+        <x:v>示例半成品</x:v>
+      </x:c>
+      <x:c r="G44" s="111" t="str">
+        <x:v>控制方式</x:v>
+      </x:c>
+      <x:c r="H44" s="111" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="125" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="B45" s="125" t="str">
+        <x:v>腐肉/骨/线/少量火药或木材</x:v>
+      </x:c>
+      <x:c r="C45" s="125" t="str">
+        <x:v>6.5%</x:v>
+      </x:c>
+      <x:c r="D45" s="125" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E45" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F45" s="125" t="str">
+        <x:v>枪管/机匣/枪托</x:v>
+      </x:c>
+      <x:c r="G45" s="125" t="str">
+        <x:v>Apocalypse Mobs 脚本</x:v>
+      </x:c>
+      <x:c r="H45" s="125" t="str"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="125" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="B46" s="125" t="str">
+        <x:v>腐肉/火药/铁粒/铜</x:v>
+      </x:c>
+      <x:c r="C46" s="125" t="str">
+        <x:v>12.5%</x:v>
+      </x:c>
+      <x:c r="D46" s="125" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E46" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F46" s="125" t="str">
+        <x:v>基础枪械半成品</x:v>
+      </x:c>
+      <x:c r="G46" s="125" t="str">
+        <x:v>Apocalypse Mobs 脚本</x:v>
+      </x:c>
+      <x:c r="H46" s="125" t="str"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="125" t="str">
+        <x:v>T3</x:v>
+      </x:c>
+      <x:c r="B47" s="125" t="str">
+        <x:v>铁锭/红石/火药/绿宝石</x:v>
+      </x:c>
+      <x:c r="C47" s="125" t="str">
+        <x:v>22.5%</x:v>
+      </x:c>
+      <x:c r="D47" s="125" t="str">
+        <x:v>0.04%</x:v>
+      </x:c>
+      <x:c r="E47" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F47" s="125" t="str">
+        <x:v>基础枪械半成品</x:v>
+      </x:c>
+      <x:c r="G47" s="125" t="str">
+        <x:v>Apocalypse Mobs 脚本</x:v>
+      </x:c>
+      <x:c r="H47" s="125" t="str"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="125" t="str">
+        <x:v>T4 精英</x:v>
+      </x:c>
+      <x:c r="B48" s="125" t="str">
+        <x:v>铁/金/红石/钻石</x:v>
+      </x:c>
+      <x:c r="C48" s="125" t="str">
+        <x:v>固定 1 件</x:v>
+      </x:c>
+      <x:c r="D48" s="125" t="str">
+        <x:v>0.15%</x:v>
+      </x:c>
+      <x:c r="E48" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F48" s="125" t="str">
+        <x:v>重型枪管/陶瓷/凯夫拉</x:v>
+      </x:c>
+      <x:c r="G48" s="125" t="str">
+        <x:v>Apocalypse Mobs 脚本</x:v>
+      </x:c>
+      <x:c r="H48" s="125" t="str"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="125" t="str">
+        <x:v>T5 母体</x:v>
+      </x:c>
+      <x:c r="B49" s="125" t="str">
+        <x:v>高价值原版材料</x:v>
+      </x:c>
+      <x:c r="C49" s="125" t="str">
+        <x:v>固定 2 件</x:v>
+      </x:c>
+      <x:c r="D49" s="125" t="str">
+        <x:v>1%</x:v>
+      </x:c>
+      <x:c r="E49" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F49" s="125" t="str">
+        <x:v>高级半成品</x:v>
+      </x:c>
+      <x:c r="G49" s="125" t="str">
+        <x:v>Apocalypse Mobs 脚本</x:v>
+      </x:c>
+      <x:c r="H49" s="125" t="str"/>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="125" t="str">
+        <x:v>Boss 文件夹</x:v>
+      </x:c>
+      <x:c r="B50" s="125" t="str">
+        <x:v>大量材料/弹药/核心</x:v>
+      </x:c>
+      <x:c r="C50" s="125" t="str">
+        <x:v>按表</x:v>
+      </x:c>
+      <x:c r="D50" s="125" t="str">
+        <x:v>1%–2%</x:v>
+      </x:c>
+      <x:c r="E50" s="125" t="str">
+        <x:v>不掉</x:v>
+      </x:c>
+      <x:c r="F50" s="125" t="str">
+        <x:v>Boss 特殊核心</x:v>
+      </x:c>
+      <x:c r="G50" s="125" t="str">
+        <x:v>Loot Table</x:v>
+      </x:c>
+      <x:c r="H50" s="125" t="str">
+        <x:v>Siren 2%；铁傀儡 1% Titan + 0.5% M82</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="125" t="str"/>
+      <x:c r="B51" s="125" t="str"/>
+      <x:c r="C51" s="125" t="str"/>
+      <x:c r="D51" s="125" t="str"/>
+      <x:c r="E51" s="125" t="str"/>
+      <x:c r="F51" s="125" t="str"/>
+      <x:c r="G51" s="125" t="str"/>
+      <x:c r="H51" s="125" t="str"/>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="111" t="str">
+        <x:v>商店类型</x:v>
+      </x:c>
+      <x:c r="B52" s="111" t="str">
+        <x:v>商品范围</x:v>
+      </x:c>
+      <x:c r="C52" s="111" t="str">
+        <x:v>回收限制</x:v>
+      </x:c>
+      <x:c r="D52" s="111" t="str">
+        <x:v>依赖</x:v>
+      </x:c>
+      <x:c r="E52" s="111" t="str"/>
+      <x:c r="F52" s="111" t="str"/>
+      <x:c r="G52" s="111" t="str"/>
+      <x:c r="H52" s="111" t="str"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="125" t="str">
+        <x:v>杂货商</x:v>
+      </x:c>
+      <x:c r="B53" s="125" t="str">
+        <x:v>食物/医疗/原版资源回收</x:v>
+      </x:c>
+      <x:c r="C53" s="125" t="str">
+        <x:v>原版物资每日收益上限 3000</x:v>
+      </x:c>
+      <x:c r="D53" s="125" t="str">
+        <x:v>SAPI 可独立运行</x:v>
+      </x:c>
+      <x:c r="E53" s="125" t="str"/>
+      <x:c r="F53" s="125" t="str"/>
+      <x:c r="G53" s="125" t="str"/>
+      <x:c r="H53" s="125" t="str"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="125" t="str">
+        <x:v>军火商</x:v>
+      </x:c>
+      <x:c r="B54" s="125" t="str">
+        <x:v>弹药/基础半成品/普通与 Rare 蓝图</x:v>
+      </x:c>
+      <x:c r="C54" s="125" t="str"/>
+      <x:c r="D54" s="125" t="str">
+        <x:v>Test Gun 可选；缺少时不扣款</x:v>
+      </x:c>
+      <x:c r="E54" s="125" t="str"/>
+      <x:c r="F54" s="125" t="str"/>
+      <x:c r="G54" s="125" t="str"/>
+      <x:c r="H54" s="125" t="str"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="125" t="str">
+        <x:v>高级军备商</x:v>
+      </x:c>
+      <x:c r="B55" s="125" t="str">
+        <x:v>限定 Epic/高级半成品/抽奖入口</x:v>
+      </x:c>
+      <x:c r="C55" s="125" t="str">
+        <x:v>限定蓝图每日 1 张</x:v>
+      </x:c>
+      <x:c r="D55" s="125" t="str">
+        <x:v>Test Gun 可选</x:v>
+      </x:c>
+      <x:c r="E55" s="125" t="str"/>
+      <x:c r="F55" s="125" t="str"/>
+      <x:c r="G55" s="125" t="str"/>
+      <x:c r="H55" s="125" t="str"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="125" t="str">
+        <x:v>载具商</x:v>
+      </x:c>
+      <x:c r="B56" s="125" t="str">
+        <x:v>载具蓝图/组件</x:v>
+      </x:c>
+      <x:c r="C56" s="125" t="str"/>
+      <x:c r="D56" s="125" t="str">
+        <x:v>Apocalypse Vehicles 可选</x:v>
+      </x:c>
+      <x:c r="E56" s="125" t="str"/>
+      <x:c r="F56" s="125" t="str"/>
+      <x:c r="G56" s="125" t="str"/>
+      <x:c r="H56" s="125" t="str"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="125" t="str"/>
+      <x:c r="B57" s="125" t="str"/>
+      <x:c r="C57" s="125" t="str"/>
+      <x:c r="D57" s="125" t="str"/>
+      <x:c r="E57" s="125" t="str"/>
+      <x:c r="F57" s="125" t="str"/>
+      <x:c r="G57" s="125" t="str"/>
+      <x:c r="H57" s="125" t="str"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="111" t="str">
+        <x:v>载具蓝图</x:v>
+      </x:c>
+      <x:c r="B58" s="111" t="str">
+        <x:v>玩家合成</x:v>
+      </x:c>
+      <x:c r="C58" s="111" t="str">
+        <x:v>NPC 价格</x:v>
+      </x:c>
+      <x:c r="D58" s="111" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+      <x:c r="E58" s="111" t="str"/>
+      <x:c r="F58" s="111" t="str"/>
+      <x:c r="G58" s="111" t="str"/>
+      <x:c r="H58" s="111" t="str"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="125" t="str">
+        <x:v>摩托车</x:v>
+      </x:c>
+      <x:c r="B59" s="126" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="C59" s="126" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D59" s="125" t="str">
+        <x:v>玩家配方</x:v>
+      </x:c>
+      <x:c r="E59" s="125" t="str"/>
+      <x:c r="F59" s="125" t="str"/>
+      <x:c r="G59" s="125" t="str"/>
+      <x:c r="H59" s="125" t="str"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="125" t="str">
+        <x:v>冲锋快艇</x:v>
+      </x:c>
+      <x:c r="B60" s="126" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="C60" s="126" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D60" s="125" t="str">
+        <x:v>玩家配方</x:v>
+      </x:c>
+      <x:c r="E60" s="125" t="str"/>
+      <x:c r="F60" s="125" t="str"/>
+      <x:c r="G60" s="125" t="str"/>
+      <x:c r="H60" s="125" t="str"/>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="125" t="str">
+        <x:v>皮卡</x:v>
+      </x:c>
+      <x:c r="B61" s="126" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C61" s="126" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="D61" s="125" t="str">
+        <x:v>载具商</x:v>
+      </x:c>
+      <x:c r="E61" s="125" t="str"/>
+      <x:c r="F61" s="125" t="str"/>
+      <x:c r="G61" s="125" t="str"/>
+      <x:c r="H61" s="125" t="str"/>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="125" t="str">
+        <x:v>救护车</x:v>
+      </x:c>
+      <x:c r="B62" s="126" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C62" s="126" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="D62" s="125" t="str">
+        <x:v>载具商</x:v>
+      </x:c>
+      <x:c r="E62" s="125" t="str"/>
+      <x:c r="F62" s="125" t="str"/>
+      <x:c r="G62" s="125" t="str"/>
+      <x:c r="H62" s="125" t="str"/>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="125" t="str">
+        <x:v>军用直升机</x:v>
+      </x:c>
+      <x:c r="B63" s="126" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="C63" s="126" t="n">
+        <x:v>80000</x:v>
+      </x:c>
+      <x:c r="D63" s="125" t="str">
+        <x:v>载具商</x:v>
+      </x:c>
+      <x:c r="E63" s="125" t="str"/>
+      <x:c r="F63" s="125" t="str"/>
+      <x:c r="G63" s="125" t="str"/>
+      <x:c r="H63" s="125" t="str"/>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="125" t="str"/>
+      <x:c r="B64" s="125" t="str"/>
+      <x:c r="C64" s="125" t="str"/>
+      <x:c r="D64" s="125" t="str"/>
+      <x:c r="E64" s="125" t="str"/>
+      <x:c r="F64" s="125" t="str"/>
+      <x:c r="G64" s="125" t="str"/>
+      <x:c r="H64" s="125" t="str"/>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="111" t="str">
+        <x:v>弹药包</x:v>
+      </x:c>
+      <x:c r="B65" s="111" t="str">
+        <x:v>数量</x:v>
+      </x:c>
+      <x:c r="C65" s="111" t="str">
+        <x:v>NPC 售价</x:v>
+      </x:c>
+      <x:c r="D65" s="111" t="str">
+        <x:v>单发折算</x:v>
+      </x:c>
+      <x:c r="E65" s="111" t="str"/>
+      <x:c r="F65" s="111" t="str"/>
+      <x:c r="G65" s="111" t="str"/>
+      <x:c r="H65" s="111" t="str"/>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="125" t="str">
+        <x:v>手枪弹</x:v>
+      </x:c>
+      <x:c r="B66" s="126" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C66" s="126" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D66" s="126" t="n">
+        <x:f>C66/B66</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E66" s="125" t="str"/>
+      <x:c r="F66" s="125" t="str"/>
+      <x:c r="G66" s="125" t="str"/>
+      <x:c r="H66" s="125" t="str"/>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="125" t="str">
+        <x:v>.45/SMG</x:v>
+      </x:c>
+      <x:c r="B67" s="126" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C67" s="126" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="D67" s="126" t="n">
+        <x:f>C67/B67</x:f>
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="E67" s="125" t="str"/>
+      <x:c r="F67" s="125" t="str"/>
+      <x:c r="G67" s="125" t="str"/>
+      <x:c r="H67" s="125" t="str"/>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="125" t="str">
+        <x:v>步枪弹</x:v>
+      </x:c>
+      <x:c r="B68" s="126" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C68" s="126" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="D68" s="126" t="n">
+        <x:f>C68/B68</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E68" s="125" t="str"/>
+      <x:c r="F68" s="125" t="str"/>
+      <x:c r="G68" s="125" t="str"/>
+      <x:c r="H68" s="125" t="str"/>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="125" t="str">
+        <x:v>霰弹</x:v>
+      </x:c>
+      <x:c r="B69" s="126" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C69" s="126" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="D69" s="126" t="n">
+        <x:f>C69/B69</x:f>
+        <x:v>18.333333333333332</x:v>
+      </x:c>
+      <x:c r="E69" s="125" t="str"/>
+      <x:c r="F69" s="125" t="str"/>
+      <x:c r="G69" s="125" t="str"/>
+      <x:c r="H69" s="125" t="str"/>
+    </x:row>
+    <x:row r="70" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A70" s="125" t="str">
+        <x:v>重机枪弹链</x:v>
+      </x:c>
+      <x:c r="B70" s="126" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C70" s="126" t="n">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="D70" s="126" t="n">
+        <x:f>C70/B70</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E70" s="125" t="str">
+        <x:v>新图标：ammo_belt_100_generated.png</x:v>
+      </x:c>
+      <x:c r="F70" s="125" t="str"/>
+      <x:c r="G70" s="125" t="str"/>
+      <x:c r="H70" s="125" t="str"/>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="125" t="str">
+        <x:v>.50</x:v>
+      </x:c>
+      <x:c r="B71" s="126" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C71" s="126" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="D71" s="126" t="n">
+        <x:f>C71/B71</x:f>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E71" s="125" t="str"/>
+      <x:c r="F71" s="125" t="str"/>
+      <x:c r="G71" s="125" t="str"/>
+      <x:c r="H71" s="125" t="str"/>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="125" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="B72" s="126" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C72" s="126" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="D72" s="126" t="n">
+        <x:f>C72/B72</x:f>
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="E72" s="125" t="str"/>
+      <x:c r="F72" s="125" t="str"/>
+      <x:c r="G72" s="125" t="str"/>
+      <x:c r="H72" s="125" t="str"/>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="125" t="str">
+        <x:v>40mm</x:v>
+      </x:c>
+      <x:c r="B73" s="126" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C73" s="126" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="D73" s="126" t="n">
+        <x:f>C73/B73</x:f>
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E73" s="125" t="str"/>
+      <x:c r="F73" s="125" t="str"/>
+      <x:c r="G73" s="125" t="str"/>
+      <x:c r="H73" s="125" t="str"/>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="125" t="str">
+        <x:v>火箭</x:v>
+      </x:c>
+      <x:c r="B74" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C74" s="126" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="D74" s="126" t="n">
+        <x:f>C74/B74</x:f>
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="E74" s="125" t="str"/>
+      <x:c r="F74" s="125" t="str"/>
+      <x:c r="G74" s="125" t="str"/>
+      <x:c r="H74" s="125" t="str"/>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="125" t="str"/>
+      <x:c r="B75" s="125" t="str"/>
+      <x:c r="C75" s="125" t="str"/>
+      <x:c r="D75" s="125" t="str"/>
+      <x:c r="E75" s="125" t="str"/>
+      <x:c r="F75" s="125" t="str"/>
+      <x:c r="G75" s="125" t="str"/>
+      <x:c r="H75" s="125" t="str"/>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="111" t="str">
+        <x:v>城市摸金箱</x:v>
+      </x:c>
+      <x:c r="B76" s="111" t="str">
+        <x:v>权重</x:v>
+      </x:c>
+      <x:c r="C76" s="111" t="str">
+        <x:v>概率</x:v>
+      </x:c>
+      <x:c r="D76" s="111" t="str">
+        <x:v>数量限制</x:v>
+      </x:c>
+      <x:c r="E76" s="111" t="str">
+        <x:v>与金币奖池关系</x:v>
+      </x:c>
+      <x:c r="F76" s="111" t="str"/>
+      <x:c r="G76" s="111" t="str"/>
+      <x:c r="H76" s="111" t="str"/>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="125" t="str">
+        <x:v>普通</x:v>
+      </x:c>
+      <x:c r="B77" s="126" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C77" s="127" t="n">
+        <x:f>B77/SUM($B$77:$B$81)</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D77" s="125" t="str">
+        <x:v>不限制</x:v>
+      </x:c>
+      <x:c r="E77" s="125" t="str">
+        <x:v>独立 Loot Table</x:v>
+      </x:c>
+      <x:c r="F77" s="125" t="str"/>
+      <x:c r="G77" s="125" t="str"/>
+      <x:c r="H77" s="125" t="str"/>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="125" t="str">
+        <x:v>精良</x:v>
+      </x:c>
+      <x:c r="B78" s="126" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C78" s="127" t="n">
+        <x:f>B78/SUM($B$77:$B$81)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="D78" s="125" t="str">
+        <x:v>不限制</x:v>
+      </x:c>
+      <x:c r="E78" s="125" t="str">
+        <x:v>独立 Loot Table</x:v>
+      </x:c>
+      <x:c r="F78" s="125" t="str"/>
+      <x:c r="G78" s="125" t="str"/>
+      <x:c r="H78" s="125" t="str"/>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="125" t="str">
+        <x:v>Epic</x:v>
+      </x:c>
+      <x:c r="B79" s="126" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C79" s="127" t="n">
+        <x:f>B79/SUM($B$77:$B$81)</x:f>
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D79" s="125" t="str">
+        <x:v>不限制</x:v>
+      </x:c>
+      <x:c r="E79" s="125" t="str">
+        <x:v>独立 Loot Table</x:v>
+      </x:c>
+      <x:c r="F79" s="125" t="str"/>
+      <x:c r="G79" s="125" t="str"/>
+      <x:c r="H79" s="125" t="str"/>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="125" t="str">
+        <x:v>Legendary</x:v>
+      </x:c>
+      <x:c r="B80" s="126" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C80" s="127" t="n">
+        <x:f>B80/SUM($B$77:$B$81)</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D80" s="125" t="str">
+        <x:v>不限制</x:v>
+      </x:c>
+      <x:c r="E80" s="125" t="str">
+        <x:v>独立 Loot Table</x:v>
+      </x:c>
+      <x:c r="F80" s="125" t="str"/>
+      <x:c r="G80" s="125" t="str"/>
+      <x:c r="H80" s="125" t="str"/>
+    </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="125" t="str">
+        <x:v>Mythic</x:v>
+      </x:c>
+      <x:c r="B81" s="126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C81" s="127" t="n">
+        <x:f>B81/SUM($B$77:$B$81)</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="D81" s="125" t="str">
+        <x:v>不限制；需要神话密钥</x:v>
+      </x:c>
+      <x:c r="E81" s="125" t="str">
+        <x:v>独立 Loot Table</x:v>
+      </x:c>
+      <x:c r="F81" s="125" t="str"/>
+      <x:c r="G81" s="125" t="str"/>
+      <x:c r="H81" s="125" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -8646,7 +10417,7 @@
         <x:v>test_gun:blueprint_pkm</x:v>
       </x:c>
       <x:c r="X19" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Y19" s="76" t="str">
         <x:v>是</x:v>
@@ -8730,7 +10501,7 @@
         <x:v>test_gun:blueprint_m1014_ward</x:v>
       </x:c>
       <x:c r="X20" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Y20" s="76" t="str">
         <x:v>是</x:v>
@@ -8810,9 +10581,11 @@
         <x:v>无</x:v>
       </x:c>
       <x:c r="V21" s="76" t="str"/>
-      <x:c r="W21" s="76"/>
+      <x:c r="W21" s="76" t="str">
+        <x:v>test_gun:blueprint_usas12</x:v>
+      </x:c>
       <x:c r="X21" s="76" t="str">
-        <x:v>不需要/未配置</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Y21" s="76" t="str">
         <x:v>是</x:v>
@@ -9062,7 +10835,7 @@
         <x:v>test_gun:blueprint_ak47_commander</x:v>
       </x:c>
       <x:c r="X24" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="Y24" s="76" t="str">
         <x:v>是</x:v>
@@ -9332,7 +11105,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20701cbc7fd24987"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cfa75726fe04e81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10942,7 +12715,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee634d6e97145cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31d06b8115a24b4c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11088,7 +12861,7 @@
         <x:v>传说</x:v>
       </x:c>
       <x:c r="D6" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E6" s="76" t="str">
         <x:v>test_gun:ak47_commander</x:v>
@@ -11097,10 +12870,10 @@
         <x:v>test_gun:ak47_commander</x:v>
       </x:c>
       <x:c r="G6" s="76" t="str">
-        <x:v>minecraft:nether_star×2; minecraft:amethyst_shard×2; test_gun:blueprint_blank×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H6" s="76" t="str">
-        <x:v>minecraft:nether_star×2; minecraft:amethyst_shard×2; minecraft:paper×1; minecraft:ink_sac×0.3333333333333333; minecraft:feather×0.3333333333333333</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I6" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/test_guns_2d_addon/test_guns_bp/items/blueprint_ak47_commander.json</x:v>
@@ -11108,7 +12881,9 @@
       <x:c r="J6" s="76" t="str">
         <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_ak47_commander.json</x:v>
       </x:c>
-      <x:c r="K6" s="77" t="str"/>
+      <x:c r="K6" s="77" t="str">
+        <x:v>Legendary 限定池；玩家不可合成</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="76" t="str">
@@ -11317,7 +13092,7 @@
         <x:v>史诗</x:v>
       </x:c>
       <x:c r="D13" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E13" s="76" t="str">
         <x:v>test_gun:flash_shield</x:v>
@@ -11326,10 +13101,10 @@
         <x:v>test_gun:flash_shield</x:v>
       </x:c>
       <x:c r="G13" s="76" t="str">
-        <x:v>minecraft:glowstone×2; minecraft:diamond×2; test_gun:blueprint_blank×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H13" s="76" t="str">
-        <x:v>minecraft:glowstone×2; minecraft:diamond×2; minecraft:paper×1; minecraft:ink_sac×0.3333333333333333; minecraft:feather×0.3333333333333333</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I13" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/test_guns_2d_addon/test_guns_bp/items/blueprint_flash_shield.json</x:v>
@@ -11337,7 +13112,9 @@
       <x:c r="J13" s="76" t="str">
         <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_flash_shield.json</x:v>
       </x:c>
-      <x:c r="K13" s="77" t="str"/>
+      <x:c r="K13" s="77" t="str">
+        <x:v>限定 Epic；高级军备商 26000 或 Epic 奖池</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="76" t="str">
@@ -11546,7 +13323,7 @@
         <x:v>史诗</x:v>
       </x:c>
       <x:c r="D20" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E20" s="76" t="str">
         <x:v>test_gun:m1014_ward</x:v>
@@ -11555,10 +13332,10 @@
         <x:v>test_gun:m1014_ward</x:v>
       </x:c>
       <x:c r="G20" s="76" t="str">
-        <x:v>test_gun:blueprint_blank×1; test_gun:part_ceramic_plate×1; minecraft:gold_ingot×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H20" s="76" t="str">
-        <x:v>minecraft:paper×1; minecraft:ink_sac×0.3333333333333333; minecraft:feather×0.3333333333333333; minecraft:iron_ingot×2; minecraft:clay_ball×2; minecraft:quartz×0.5; minecraft:gold_ingot×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I20" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/test_guns_2d_addon/test_guns_bp/items/blueprint_m1014_ward.json</x:v>
@@ -11566,7 +13343,9 @@
       <x:c r="J20" s="76" t="str">
         <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_m1014_ward.json</x:v>
       </x:c>
-      <x:c r="K20" s="77" t="str"/>
+      <x:c r="K20" s="77" t="str">
+        <x:v>限定 Epic；高级军备商 28000 或 Epic 奖池</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="76" t="str">
@@ -11806,7 +13585,7 @@
         <x:v>史诗</x:v>
       </x:c>
       <x:c r="D28" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E28" s="76" t="str">
         <x:v>test_gun:pkm</x:v>
@@ -11815,10 +13594,10 @@
         <x:v>test_gun:pkm</x:v>
       </x:c>
       <x:c r="G28" s="76" t="str">
-        <x:v>test_gun:blueprint_blank×1; minecraft:iron_block×1; minecraft:blaze_rod×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H28" s="76" t="str">
-        <x:v>minecraft:paper×1; minecraft:ink_sac×0.3333333333333333; minecraft:feather×0.3333333333333333; minecraft:iron_block×1; minecraft:blaze_rod×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I28" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/test_guns_2d_addon/test_guns_bp/items/blueprint_pkm.json</x:v>
@@ -11826,7 +13605,9 @@
       <x:c r="J28" s="76" t="str">
         <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_pkm.json</x:v>
       </x:c>
-      <x:c r="K28" s="77" t="str"/>
+      <x:c r="K28" s="77" t="str">
+        <x:v>限定 Epic；高级军备商 30000 或 Epic 奖池</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="76" t="str">
@@ -12004,7 +13785,7 @@
         <x:v>史诗</x:v>
       </x:c>
       <x:c r="D34" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E34" s="76" t="str">
         <x:v>test_gun:titan_chest</x:v>
@@ -12013,10 +13794,10 @@
         <x:v>test_gun:armor_titan_chest</x:v>
       </x:c>
       <x:c r="G34" s="76" t="str">
-        <x:v>test_gun:blueprint_blank×1; minecraft:diamond×1; minecraft:netherite_scrap×1; minecraft:amethyst_shard×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H34" s="76" t="str">
-        <x:v>minecraft:paper×1; minecraft:ink_sac×0.3333333333333333; minecraft:feather×0.3333333333333333; minecraft:diamond×1; minecraft:netherite_scrap×1; minecraft:amethyst_shard×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I34" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/test_guns_2d_addon/test_guns_bp/items/blueprint_titan_chest.json</x:v>
@@ -12024,7 +13805,9 @@
       <x:c r="J34" s="76" t="str">
         <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_titan_chest.json</x:v>
       </x:c>
-      <x:c r="K34" s="77" t="str"/>
+      <x:c r="K34" s="77" t="str">
+        <x:v>限定 Epic；高级军备商 36000 或 Epic 奖池</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="76" t="str">
@@ -12104,7 +13887,7 @@
         <x:v>未标注</x:v>
       </x:c>
       <x:c r="D37" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E37" s="76" t="str">
         <x:v>survival_vehicle:ambulance</x:v>
@@ -12113,10 +13896,10 @@
         <x:v>ab_ve:ambulance_spawner</x:v>
       </x:c>
       <x:c r="G37" s="76" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:glistering_melon_slice×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H37" s="76" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:glistering_melon_slice×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I37" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_ambulance.json</x:v>
@@ -12124,7 +13907,9 @@
       <x:c r="J37" s="76" t="str">
         <x:v>apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_ambulance.json</x:v>
       </x:c>
-      <x:c r="K37" s="77" t="str"/>
+      <x:c r="K37" s="77" t="str">
+        <x:v>载具商 40000；玩家不可合成</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="76" t="str">
@@ -12138,7 +13923,7 @@
         <x:v>精良</x:v>
       </x:c>
       <x:c r="D38" s="76" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E38" s="76" t="str">
         <x:v>survival_vehicle:helicopter</x:v>
@@ -12147,10 +13932,10 @@
         <x:v>ab_ve:helicopter_spawner</x:v>
       </x:c>
       <x:c r="G38" s="76" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:redstone_block×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H38" s="76" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:redstone_block×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I38" s="76" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_helicopter.json</x:v>
@@ -12158,7 +13943,9 @@
       <x:c r="J38" s="76" t="str">
         <x:v>apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_helicopter.json</x:v>
       </x:c>
-      <x:c r="K38" s="77" t="str"/>
+      <x:c r="K38" s="77" t="str">
+        <x:v>载具商 80000；玩家不可合成</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="76" t="str">
@@ -12240,7 +14027,7 @@
         <x:v>未标注</x:v>
       </x:c>
       <x:c r="D41" s="81" t="str">
-        <x:v>是</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="E41" s="81" t="str">
         <x:v>survival_vehicle:truck</x:v>
@@ -12249,10 +14036,10 @@
         <x:v>ab_ve:truck_spawner</x:v>
       </x:c>
       <x:c r="G41" s="81" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:chest×1</x:v>
+        <x:v>无（掉落/商店/奖池来源）</x:v>
       </x:c>
       <x:c r="H41" s="81" t="str">
-        <x:v>minecraft:compass×1; minecraft:redstone×2; minecraft:paper×1; minecraft:chest×1</x:v>
+        <x:v>不适用</x:v>
       </x:c>
       <x:c r="I41" s="81" t="str">
         <x:v>https://github.com/GallonHong/lotm-mc/blob/f383d05769b1a71b5bb939f506c57b7c6821261d/apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_truck.json</x:v>
@@ -12260,7 +14047,42 @@
       <x:c r="J41" s="81" t="str">
         <x:v>apocalypse_vehicles_addon/apocalypse_vehicles_bp/items/blueprints/blueprint_truck.json</x:v>
       </x:c>
-      <x:c r="K41" s="82" t="str"/>
+      <x:c r="K41" s="82" t="str">
+        <x:v>载具商 25000；玩家不可合成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>test_gun:blueprint_usas12</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>USAS-12 嗜血狂潮设计图 [史诗·不可合成]</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>史诗</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>test_gun:usas12</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>test_gun:usas12</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>无（NPC/Epic 奖池）</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="I42" t="str"/>
+      <x:c r="J42" t="str">
+        <x:v>test_guns_2d_addon/test_guns_bp/items/blueprint_usas12.json</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
+        <x:v>高级军备商 32000；Epic 奖池限定蓝图</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -12270,7 +14092,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5caf06dbf05c44a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c08165e7054d40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14869,7 +16691,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddd1e0722b3f40a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c412d8b143f4519"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19993,7 +21815,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c90ac5e94547bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd90a84494a794950"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35573,7 +37395,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a84c0c2de5c4a99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b86be2ba8494469"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35930,7 +37752,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb545c7363bde4fcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2e8bce7d1724670"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37668,7 +39490,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0bcb7db428e4e5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98ff48c413604ebe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>